<commit_message>
Remove internal capture-channel assignments from public snapshot
</commit_message>
<xml_diff>
--- a/reports/Zeekr_X_CAN_Matrix_EN.xlsx
+++ b/reports/Zeekr_X_CAN_Matrix_EN.xlsx
@@ -211,17 +211,16 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="T11" displayName="T11" ref="A1:H111" headerRowCount="1">
-  <autoFilter ref="A1:H111"/>
-  <tableColumns count="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="T11" displayName="T11" ref="A1:G111" headerRowCount="1">
+  <autoFilter ref="A1:G111"/>
+  <tableColumns count="7">
     <tableColumn id="1" name="Experiment"/>
     <tableColumn id="2" name="Source_ECU"/>
-    <tableColumn id="3" name="ECU_Channel"/>
-    <tableColumn id="4" name="CAN_ID"/>
-    <tableColumn id="5" name="Count"/>
-    <tableColumn id="6" name="Median_Interval_ms"/>
-    <tableColumn id="7" name="Unique_Payloads"/>
-    <tableColumn id="8" name="Trace_Reference"/>
+    <tableColumn id="3" name="CAN_ID"/>
+    <tableColumn id="4" name="Count"/>
+    <tableColumn id="5" name="Median_Interval_ms"/>
+    <tableColumn id="6" name="Unique_Payloads"/>
+    <tableColumn id="7" name="Trace_Reference"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -1018,17 +1017,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H111"/>
+  <dimension ref="A1:G111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="17" customWidth="1" min="7" max="7"/>
-    <col width="65" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="65" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1044,30 +1042,25 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>ECU_Channel</t>
+          <t>CAN_ID</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>CAN_ID</t>
+          <t>Count</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Count</t>
+          <t>Median_Interval_ms</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Median_Interval_ms</t>
+          <t>Unique_Payloads</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Unique_Payloads</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Trace_Reference</t>
         </is>
@@ -1086,30 +1079,25 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
+          <t>0x15</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>7968</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>9.999000000000535</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>0x15</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>7968</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>9.999000000000535</t>
-        </is>
-      </c>
       <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>sha256:5a826e4d3e2e20c2d978076219c097f79d4bbc1a048489617512a5944bb9eeb0:line:34</t>
         </is>
@@ -1128,30 +1116,25 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x31</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>0x31</t>
+          <t>5312</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>5312</t>
+          <t>14.995999999996457</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>14.995999999996457</t>
+          <t>33</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>33</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>sha256:5a826e4d3e2e20c2d978076219c097f79d4bbc1a048489617512a5944bb9eeb0:line:36</t>
         </is>
@@ -1170,30 +1153,25 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x3A</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>0x3A</t>
+          <t>7969</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>7969</t>
+          <t>9.993000000008578</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>9.993000000008578</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>32</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>sha256:5a826e4d3e2e20c2d978076219c097f79d4bbc1a048489617512a5944bb9eeb0:line:11</t>
         </is>
@@ -1212,30 +1190,25 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
+          <t>0x47</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>7969</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>9.994999999996423</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>0x47</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>7969</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>9.994999999996423</t>
-        </is>
-      </c>
       <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>sha256:5a826e4d3e2e20c2d978076219c097f79d4bbc1a048489617512a5944bb9eeb0:line:9</t>
         </is>
@@ -1254,30 +1227,25 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x4A</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>0x4A</t>
+          <t>7968</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>7968</t>
+          <t>9.988000000006991</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>9.988000000006991</t>
+          <t>15</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>sha256:5a826e4d3e2e20c2d978076219c097f79d4bbc1a048489617512a5944bb9eeb0:line:32</t>
         </is>
@@ -1296,30 +1264,25 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x4B</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>0x4B</t>
+          <t>7968</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>7968</t>
+          <t>9.995000000003529</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>9.995000000003529</t>
+          <t>15</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>sha256:5a826e4d3e2e20c2d978076219c097f79d4bbc1a048489617512a5944bb9eeb0:line:37</t>
         </is>
@@ -1338,30 +1301,25 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x50</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>0x50</t>
+          <t>7969</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>7969</t>
+          <t>9.995000000003529</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>9.995000000003529</t>
+          <t>15</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>sha256:5a826e4d3e2e20c2d978076219c097f79d4bbc1a048489617512a5944bb9eeb0:line:12</t>
         </is>
@@ -1380,30 +1338,25 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x56</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>0x56</t>
+          <t>5313</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>5313</t>
+          <t>14.998999999988882</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>14.998999999988882</t>
+          <t>45</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>45</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>sha256:5a826e4d3e2e20c2d978076219c097f79d4bbc1a048489617512a5944bb9eeb0:line:13</t>
         </is>
@@ -1422,30 +1375,25 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x66</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>0x66</t>
+          <t>5312</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>5312</t>
+          <t>15.001999999995519</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>15.001999999995519</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>sha256:5a826e4d3e2e20c2d978076219c097f79d4bbc1a048489617512a5944bb9eeb0:line:54</t>
         </is>
@@ -1464,30 +1412,25 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x71</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>0x71</t>
+          <t>5312</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>5312</t>
+          <t>15.000999999998044</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>15.000999999998044</t>
+          <t>14</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>sha256:5a826e4d3e2e20c2d978076219c097f79d4bbc1a048489617512a5944bb9eeb0:line:55</t>
         </is>
@@ -1506,30 +1449,25 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x81</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>0x81</t>
+          <t>400</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>14.990999999998422</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>14.990999999998422</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>sha256:5a826e4d3e2e20c2d978076219c097f79d4bbc1a048489617512a5944bb9eeb0:line:56</t>
         </is>
@@ -1548,30 +1486,25 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x84</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>0x84</t>
+          <t>3187</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>3187</t>
+          <t>25.003999999999138</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>25.003999999999138</t>
+          <t>104</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>104</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>sha256:5a826e4d3e2e20c2d978076219c097f79d4bbc1a048489617512a5944bb9eeb0:line:95</t>
         </is>
@@ -1590,30 +1523,25 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x86</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>0x86</t>
+          <t>5312</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>5312</t>
+          <t>15.00499999999505</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>15.00499999999505</t>
+          <t>14</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>sha256:5a826e4d3e2e20c2d978076219c097f79d4bbc1a048489617512a5944bb9eeb0:line:57</t>
         </is>
@@ -1632,30 +1560,25 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x103</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>0x103</t>
+          <t>3984</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>3984</t>
+          <t>19.992000000002008</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>19.992000000002008</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>sha256:5a826e4d3e2e20c2d978076219c097f79d4bbc1a048489617512a5944bb9eeb0:line:74</t>
         </is>
@@ -1674,30 +1597,25 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x116</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>0x116</t>
+          <t>3984</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>3984</t>
+          <t>19.997000000003595</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>19.997000000003595</t>
+          <t>74</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>74</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>sha256:5a826e4d3e2e20c2d978076219c097f79d4bbc1a048489617512a5944bb9eeb0:line:39</t>
         </is>
@@ -1716,30 +1634,25 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x131</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>0x131</t>
+          <t>3984</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>3984</t>
+          <t>19.99599999999191</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>19.99599999999191</t>
+          <t>104</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>104</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>sha256:5a826e4d3e2e20c2d978076219c097f79d4bbc1a048489617512a5944bb9eeb0:line:40</t>
         </is>
@@ -1758,30 +1671,25 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
+          <t>0x138</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>240</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>24.856999999997242</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>0x138</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>240</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>24.856999999997242</t>
-        </is>
-      </c>
       <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>sha256:5a826e4d3e2e20c2d978076219c097f79d4bbc1a048489617512a5944bb9eeb0:line:96</t>
         </is>
@@ -1800,30 +1708,25 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x148</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>0x148</t>
+          <t>3187</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>3187</t>
+          <t>24.98549999999966</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>24.98549999999966</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="inlineStr">
         <is>
           <t>sha256:5a826e4d3e2e20c2d978076219c097f79d4bbc1a048489617512a5944bb9eeb0:line:97</t>
         </is>
@@ -1842,30 +1745,25 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x151</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>0x151</t>
+          <t>2656</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>2656</t>
+          <t>30.000000000001137</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>30.000000000001137</t>
+          <t>162</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
-        <is>
-          <t>162</t>
-        </is>
-      </c>
-      <c r="H20" s="2" t="inlineStr">
         <is>
           <t>sha256:5a826e4d3e2e20c2d978076219c097f79d4bbc1a048489617512a5944bb9eeb0:line:98</t>
         </is>
@@ -1884,30 +1782,25 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x155</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>0x155</t>
+          <t>3188</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>3188</t>
+          <t>24.96200000000215</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>24.96200000000215</t>
+          <t>15</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="inlineStr">
         <is>
           <t>sha256:5a826e4d3e2e20c2d978076219c097f79d4bbc1a048489617512a5944bb9eeb0:line:14</t>
         </is>
@@ -1926,30 +1819,25 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x161</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>0x161</t>
+          <t>3187</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>3187</t>
+          <t>24.954000000004584</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>24.954000000004584</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr">
         <is>
           <t>sha256:5a826e4d3e2e20c2d978076219c097f79d4bbc1a048489617512a5944bb9eeb0:line:75</t>
         </is>
@@ -1968,30 +1856,25 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x162</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>0x162</t>
+          <t>1593</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>1593</t>
+          <t>49.98149999999768</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>49.98149999999768</t>
+          <t>1195</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
-        <is>
-          <t>1195</t>
-        </is>
-      </c>
-      <c r="H23" s="2" t="inlineStr">
         <is>
           <t>sha256:5a826e4d3e2e20c2d978076219c097f79d4bbc1a048489617512a5944bb9eeb0:line:141</t>
         </is>
@@ -2010,30 +1893,25 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x171</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>0x171</t>
+          <t>1594</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>1594</t>
+          <t>50.142999999998494</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>50.142999999998494</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="inlineStr">
         <is>
           <t>sha256:5a826e4d3e2e20c2d978076219c097f79d4bbc1a048489617512a5944bb9eeb0:line:15</t>
         </is>
@@ -2052,30 +1930,25 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x179</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>0x179</t>
+          <t>797</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>797</t>
+          <t>99.78750000000325</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>99.78750000000325</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H25" s="2" t="inlineStr">
         <is>
           <t>sha256:5a826e4d3e2e20c2d978076219c097f79d4bbc1a048489617512a5944bb9eeb0:line:166</t>
         </is>
@@ -2094,30 +1967,25 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x188</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>0x188</t>
+          <t>1139</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>1139</t>
+          <t>69.92099999999724</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>69.92099999999724</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H26" s="2" t="inlineStr">
         <is>
           <t>sha256:5a826e4d3e2e20c2d978076219c097f79d4bbc1a048489617512a5944bb9eeb0:line:17</t>
         </is>
@@ -2136,30 +2004,25 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x191</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>0x191</t>
+          <t>1139</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>1139</t>
+          <t>69.93350000000298</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>69.93350000000298</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H27" s="2" t="inlineStr">
         <is>
           <t>sha256:5a826e4d3e2e20c2d978076219c097f79d4bbc1a048489617512a5944bb9eeb0:line:58</t>
         </is>
@@ -2178,30 +2041,25 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x196</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>0x196</t>
+          <t>1138</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>1138</t>
+          <t>70.00299999999982</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>70.00299999999982</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr">
         <is>
           <t>sha256:5a826e4d3e2e20c2d978076219c097f79d4bbc1a048489617512a5944bb9eeb0:line:256</t>
         </is>
@@ -2220,30 +2078,25 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x235</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>0x235</t>
+          <t>620</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>620</t>
+          <t>125.11699999999593</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>125.11699999999593</t>
+          <t>72</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
-        <is>
-          <t>72</t>
-        </is>
-      </c>
-      <c r="H29" s="2" t="inlineStr">
         <is>
           <t>sha256:5a826e4d3e2e20c2d978076219c097f79d4bbc1a048489617512a5944bb9eeb0:line:142</t>
         </is>
@@ -2262,30 +2115,25 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x236</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>0x236</t>
+          <t>610</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>610</t>
+          <t>125.14400000000592</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>125.14400000000592</t>
+          <t>72</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
-        <is>
-          <t>72</t>
-        </is>
-      </c>
-      <c r="H30" s="2" t="inlineStr">
         <is>
           <t>sha256:5a826e4d3e2e20c2d978076219c097f79d4bbc1a048489617512a5944bb9eeb0:line:184</t>
         </is>
@@ -2304,30 +2152,25 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
+          <t>0x255</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>996</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>80.06600000000219</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>0x255</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>996</t>
-        </is>
-      </c>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t>80.06600000000219</t>
-        </is>
-      </c>
       <c r="G31" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="H31" s="2" t="inlineStr">
         <is>
           <t>sha256:5a826e4d3e2e20c2d978076219c097f79d4bbc1a048489617512a5944bb9eeb0:line:100</t>
         </is>
@@ -2346,30 +2189,25 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
+          <t>0x261</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>996</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>80.09500000000003</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>0x261</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>996</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>80.09500000000003</t>
-        </is>
-      </c>
       <c r="G32" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="H32" s="2" t="inlineStr">
         <is>
           <t>sha256:5a826e4d3e2e20c2d978076219c097f79d4bbc1a048489617512a5944bb9eeb0:line:237</t>
         </is>
@@ -2388,30 +2226,25 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
+          <t>0x279</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>797</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>99.98449999999792</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>0x279</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>797</t>
-        </is>
-      </c>
-      <c r="F33" s="2" t="inlineStr">
-        <is>
-          <t>99.98449999999792</t>
-        </is>
-      </c>
       <c r="G33" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="H33" s="2" t="inlineStr">
         <is>
           <t>sha256:5a826e4d3e2e20c2d978076219c097f79d4bbc1a048489617512a5944bb9eeb0:line:167</t>
         </is>
@@ -2430,30 +2263,25 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x27A</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>0x27A</t>
+          <t>797</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>797</t>
+          <t>100.00200000000348</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>100.00200000000348</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H34" s="2" t="inlineStr">
         <is>
           <t>sha256:5a826e4d3e2e20c2d978076219c097f79d4bbc1a048489617512a5944bb9eeb0:line:185</t>
         </is>
@@ -2472,30 +2300,25 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x285</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>0x285</t>
+          <t>398</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>398</t>
+          <t>199.99600000001294</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>199.99600000001294</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H35" s="2" t="inlineStr">
         <is>
           <t>sha256:5a826e4d3e2e20c2d978076219c097f79d4bbc1a048489617512a5944bb9eeb0:line:510</t>
         </is>
@@ -2514,30 +2337,25 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x287</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>0x287</t>
+          <t>266</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>266</t>
+          <t>300.00499999999874</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>300.00499999999874</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="H36" s="2" t="inlineStr">
         <is>
           <t>sha256:5a826e4d3e2e20c2d978076219c097f79d4bbc1a048489617512a5944bb9eeb0:line:579</t>
         </is>
@@ -2556,30 +2374,25 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x289</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>0x289</t>
+          <t>797</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>797</t>
+          <t>99.86099999999709</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>99.86099999999709</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H37" s="2" t="inlineStr">
         <is>
           <t>sha256:5a826e4d3e2e20c2d978076219c097f79d4bbc1a048489617512a5944bb9eeb0:line:219</t>
         </is>
@@ -2598,30 +2411,25 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x29B</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>0x29B</t>
+          <t>2656</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>2656</t>
+          <t>29.9930000000046</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>29.9930000000046</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="H38" s="2" t="inlineStr">
         <is>
           <t>sha256:5a826e4d3e2e20c2d978076219c097f79d4bbc1a048489617512a5944bb9eeb0:line:101</t>
         </is>
@@ -2640,30 +2448,25 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x300</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>0x300</t>
+          <t>532</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>532</t>
+          <t>150.006999999988</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>150.006999999988</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H39" s="2" t="inlineStr">
         <is>
           <t>sha256:5a826e4d3e2e20c2d978076219c097f79d4bbc1a048489617512a5944bb9eeb0:line:102</t>
         </is>
@@ -2682,30 +2485,25 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x330</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>0x330</t>
+          <t>23</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>260.14499999999964</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>260.14499999999964</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H40" s="2" t="inlineStr">
         <is>
           <t>sha256:5a826e4d3e2e20c2d978076219c097f79d4bbc1a048489617512a5944bb9eeb0:line:705</t>
         </is>
@@ -2724,30 +2522,25 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x333</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>0x333</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1000.1899999999999</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>1000.1899999999999</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H41" s="2" t="inlineStr">
         <is>
           <t>sha256:5a826e4d3e2e20c2d978076219c097f79d4bbc1a048489617512a5944bb9eeb0:line:3215</t>
         </is>
@@ -2766,30 +2559,25 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x41B</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>0x41B</t>
+          <t>159</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>159</t>
+          <t>500.0084999999963</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>500.0084999999963</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H42" s="2" t="inlineStr">
         <is>
           <t>sha256:5a826e4d3e2e20c2d978076219c097f79d4bbc1a048489617512a5944bb9eeb0:line:1265</t>
         </is>
@@ -2808,30 +2596,25 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x477</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>0x477</t>
+          <t>50</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>120.00400000000155</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>120.00400000000155</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="H43" s="2" t="inlineStr">
         <is>
           <t>sha256:5a826e4d3e2e20c2d978076219c097f79d4bbc1a048489617512a5944bb9eeb0:line:186</t>
         </is>
@@ -2850,30 +2633,25 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x490</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>0x490</t>
+          <t>80</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>999.8499999999985</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>999.8499999999985</t>
+          <t>8</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="H44" s="2" t="inlineStr">
         <is>
           <t>sha256:5a826e4d3e2e20c2d978076219c097f79d4bbc1a048489617512a5944bb9eeb0:line:168</t>
         </is>
@@ -2892,30 +2670,25 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x492</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>0x492</t>
+          <t>80</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>1000.0270000000029</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>1000.0270000000029</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H45" s="2" t="inlineStr">
         <is>
           <t>sha256:5a826e4d3e2e20c2d978076219c097f79d4bbc1a048489617512a5944bb9eeb0:line:126</t>
         </is>
@@ -2934,30 +2707,25 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x526</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>0x526</t>
+          <t>99</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>1000.0154999999928</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>1000.0154999999928</t>
+          <t>7</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="H46" s="2" t="inlineStr">
         <is>
           <t>sha256:5a826e4d3e2e20c2d978076219c097f79d4bbc1a048489617512a5944bb9eeb0:line:2693</t>
         </is>
@@ -2976,30 +2744,25 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x5FA</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>0x5FA</t>
+          <t>7969</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>7969</t>
+          <t>10.00099999998838</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>10.00099999998838</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="H47" s="2" t="inlineStr">
         <is>
           <t>sha256:5a826e4d3e2e20c2d978076219c097f79d4bbc1a048489617512a5944bb9eeb0:line:41</t>
         </is>
@@ -3018,30 +2781,25 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x53</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>0x53</t>
+          <t>876</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>876</t>
+          <t>100.01100000000918</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>100.01100000000918</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H48" s="2" t="inlineStr">
         <is>
           <t>sha256:89e1fdf6f94b3a3a9f3488943c2f691ede0159f2325957178723a3ae2807e183:line:265</t>
         </is>
@@ -3060,30 +2818,25 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x141</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>0x141</t>
+          <t>4381</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>4381</t>
+          <t>20.001000000004154</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>20.001000000004154</t>
+          <t>105</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
-        <is>
-          <t>105</t>
-        </is>
-      </c>
-      <c r="H49" s="2" t="inlineStr">
         <is>
           <t>sha256:89e1fdf6f94b3a3a9f3488943c2f691ede0159f2325957178723a3ae2807e183:line:55</t>
         </is>
@@ -3102,30 +2855,25 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x142</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>0x142</t>
+          <t>2920</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>2920</t>
+          <t>29.998000000002634</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>29.998000000002634</t>
+          <t>1358</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
-        <is>
-          <t>1358</t>
-        </is>
-      </c>
-      <c r="H50" s="2" t="inlineStr">
         <is>
           <t>sha256:89e1fdf6f94b3a3a9f3488943c2f691ede0159f2325957178723a3ae2807e183:line:88</t>
         </is>
@@ -3144,30 +2892,25 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x143</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>0x143</t>
+          <t>4381</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>4381</t>
+          <t>20.008000000004245</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>20.008000000004245</t>
+          <t>365</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
-        <is>
-          <t>365</t>
-        </is>
-      </c>
-      <c r="H51" s="2" t="inlineStr">
         <is>
           <t>sha256:89e1fdf6f94b3a3a9f3488943c2f691ede0159f2325957178723a3ae2807e183:line:56</t>
         </is>
@@ -3186,30 +2929,25 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x145</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>0x145</t>
+          <t>876</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>876</t>
+          <t>100.00399999998422</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>100.00399999998422</t>
+          <t>341</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
-        <is>
-          <t>341</t>
-        </is>
-      </c>
-      <c r="H52" s="2" t="inlineStr">
         <is>
           <t>sha256:89e1fdf6f94b3a3a9f3488943c2f691ede0159f2325957178723a3ae2807e183:line:268</t>
         </is>
@@ -3228,30 +2966,25 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x175</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>0x175</t>
+          <t>876</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>876</t>
+          <t>100.01100000000207</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>100.01100000000207</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H53" s="2" t="inlineStr">
         <is>
           <t>sha256:89e1fdf6f94b3a3a9f3488943c2f691ede0159f2325957178723a3ae2807e183:line:269</t>
         </is>
@@ -3270,30 +3003,25 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x178</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>0x178</t>
+          <t>1251</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>1251</t>
+          <t>70.08150000000057</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>70.08150000000057</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="H54" s="2" t="inlineStr">
         <is>
           <t>sha256:89e1fdf6f94b3a3a9f3488943c2f691ede0159f2325957178723a3ae2807e183:line:230</t>
         </is>
@@ -3312,30 +3040,25 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x17B</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>0x17B</t>
+          <t>1752</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>1752</t>
+          <t>50.322999999998785</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>50.322999999998785</t>
+          <t>20</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="H55" s="2" t="inlineStr">
         <is>
           <t>sha256:89e1fdf6f94b3a3a9f3488943c2f691ede0159f2325957178723a3ae2807e183:line:89</t>
         </is>
@@ -3354,30 +3077,25 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x182</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>0x182</t>
+          <t>1252</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>1252</t>
+          <t>70.01400000000046</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>70.01400000000046</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H56" s="2" t="inlineStr">
         <is>
           <t>sha256:89e1fdf6f94b3a3a9f3488943c2f691ede0159f2325957178723a3ae2807e183:line:161</t>
         </is>
@@ -3396,30 +3114,25 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x18A</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>0x18A</t>
+          <t>876</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>876</t>
+          <t>100.07000000000232</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>100.07000000000232</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H57" s="2" t="inlineStr">
         <is>
           <t>sha256:89e1fdf6f94b3a3a9f3488943c2f691ede0159f2325957178723a3ae2807e183:line:272</t>
         </is>
@@ -3438,30 +3151,25 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x286</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>0x286</t>
+          <t>625</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>625</t>
+          <t>140.01900000000944</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>140.01900000000944</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="H58" s="2" t="inlineStr">
         <is>
           <t>sha256:89e1fdf6f94b3a3a9f3488943c2f691ede0159f2325957178723a3ae2807e183:line:487</t>
         </is>
@@ -3480,30 +3188,25 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x288</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>0x288</t>
+          <t>876</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>876</t>
+          <t>100.17700000000218</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>100.17700000000218</t>
+          <t>8</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="H59" s="2" t="inlineStr">
         <is>
           <t>sha256:89e1fdf6f94b3a3a9f3488943c2f691ede0159f2325957178723a3ae2807e183:line:296</t>
         </is>
@@ -3522,30 +3225,25 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x290</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>0x290</t>
+          <t>876</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>876</t>
+          <t>100.03599999998869</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>100.03599999998869</t>
+          <t>21</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
-      </c>
-      <c r="H60" s="2" t="inlineStr">
         <is>
           <t>sha256:89e1fdf6f94b3a3a9f3488943c2f691ede0159f2325957178723a3ae2807e183:line:298</t>
         </is>
@@ -3564,30 +3262,25 @@
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x293</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>0x293</t>
+          <t>219</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>219</t>
+          <t>400.143000000007</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>400.143000000007</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H61" s="2" t="inlineStr">
         <is>
           <t>sha256:89e1fdf6f94b3a3a9f3488943c2f691ede0159f2325957178723a3ae2807e183:line:667</t>
         </is>
@@ -3606,30 +3299,25 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x295</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>0x295</t>
+          <t>146</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>600.0160000000037</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>600.0160000000037</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H62" s="2" t="inlineStr">
         <is>
           <t>sha256:89e1fdf6f94b3a3a9f3488943c2f691ede0159f2325957178723a3ae2807e183:line:668</t>
         </is>
@@ -3648,30 +3336,25 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x296</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>0x296</t>
+          <t>146</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>600.0310000000013</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>600.0310000000013</t>
+          <t>60</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-      <c r="H63" s="2" t="inlineStr">
         <is>
           <t>sha256:89e1fdf6f94b3a3a9f3488943c2f691ede0159f2325957178723a3ae2807e183:line:669</t>
         </is>
@@ -3690,30 +3373,25 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x298</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>0x298</t>
+          <t>146</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>600.0329999999963</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>600.0329999999963</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="H64" s="2" t="inlineStr">
         <is>
           <t>sha256:89e1fdf6f94b3a3a9f3488943c2f691ede0159f2325957178723a3ae2807e183:line:671</t>
         </is>
@@ -3732,30 +3410,25 @@
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x301</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>0x301</t>
+          <t>146</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>600.0360000000029</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>600.0360000000029</t>
+          <t>136</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
-        <is>
-          <t>136</t>
-        </is>
-      </c>
-      <c r="H65" s="2" t="inlineStr">
         <is>
           <t>sha256:89e1fdf6f94b3a3a9f3488943c2f691ede0159f2325957178723a3ae2807e183:line:672</t>
         </is>
@@ -3774,30 +3447,25 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x310</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>0x310</t>
+          <t>219</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>219</t>
+          <t>399.98399999999634</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>399.98399999999634</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H66" s="2" t="inlineStr">
         <is>
           <t>sha256:89e1fdf6f94b3a3a9f3488943c2f691ede0159f2325957178723a3ae2807e183:line:673</t>
         </is>
@@ -3816,30 +3484,25 @@
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x315</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>0x315</t>
+          <t>109</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>109</t>
+          <t>800.9114999999998</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>800.9114999999998</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="H67" s="2" t="inlineStr">
         <is>
           <t>sha256:89e1fdf6f94b3a3a9f3488943c2f691ede0159f2325957178723a3ae2807e183:line:2115</t>
         </is>
@@ -3858,30 +3521,25 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x316</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>0x316</t>
+          <t>351</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>351</t>
+          <t>250.0440000000026</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>250.0440000000026</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H68" s="2" t="inlineStr">
         <is>
           <t>sha256:89e1fdf6f94b3a3a9f3488943c2f691ede0159f2325957178723a3ae2807e183:line:300</t>
         </is>
@@ -3900,30 +3558,25 @@
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x331</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>0x331</t>
+          <t>88</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>999.5790000000113</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>999.5790000000113</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="H69" s="2" t="inlineStr">
         <is>
           <t>sha256:89e1fdf6f94b3a3a9f3488943c2f691ede0159f2325957178723a3ae2807e183:line:2117</t>
         </is>
@@ -3942,30 +3595,25 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
+          <t>0x341</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>88</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>999.284000000003</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="D70" s="2" t="inlineStr">
-        <is>
-          <t>0x341</t>
-        </is>
-      </c>
-      <c r="E70" s="2" t="inlineStr">
-        <is>
-          <t>88</t>
-        </is>
-      </c>
-      <c r="F70" s="2" t="inlineStr">
-        <is>
-          <t>999.284000000003</t>
-        </is>
-      </c>
       <c r="G70" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="H70" s="2" t="inlineStr">
         <is>
           <t>sha256:89e1fdf6f94b3a3a9f3488943c2f691ede0159f2325957178723a3ae2807e183:line:2118</t>
         </is>
@@ -3984,30 +3632,25 @@
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x342</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>0x342</t>
+          <t>88</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>1000.0689999999963</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>1000.0689999999963</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H71" s="2" t="inlineStr">
         <is>
           <t>sha256:89e1fdf6f94b3a3a9f3488943c2f691ede0159f2325957178723a3ae2807e183:line:2120</t>
         </is>
@@ -4026,30 +3669,25 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x345</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>0x345</t>
+          <t>88</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>1000.0390000000152</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>1000.0390000000152</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H72" s="2" t="inlineStr">
         <is>
           <t>sha256:89e1fdf6f94b3a3a9f3488943c2f691ede0159f2325957178723a3ae2807e183:line:1991</t>
         </is>
@@ -4068,30 +3706,25 @@
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x346</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>0x346</t>
+          <t>88</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>1000.0919999999951</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>1000.0919999999951</t>
+          <t>59</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
-        <is>
-          <t>59</t>
-        </is>
-      </c>
-      <c r="H73" s="2" t="inlineStr">
         <is>
           <t>sha256:89e1fdf6f94b3a3a9f3488943c2f691ede0159f2325957178723a3ae2807e183:line:2121</t>
         </is>
@@ -4110,30 +3743,25 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x347</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>0x347</t>
+          <t>88</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>1000.0870000000077</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>1000.0870000000077</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="H74" s="2" t="inlineStr">
         <is>
           <t>sha256:89e1fdf6f94b3a3a9f3488943c2f691ede0159f2325957178723a3ae2807e183:line:2122</t>
         </is>
@@ -4152,30 +3780,25 @@
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x478</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>0x478</t>
+          <t>88</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>1000.0869999999935</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>1000.0869999999935</t>
+          <t>8</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="H75" s="2" t="inlineStr">
         <is>
           <t>sha256:89e1fdf6f94b3a3a9f3488943c2f691ede0159f2325957178723a3ae2807e183:line:2124</t>
         </is>
@@ -4194,30 +3817,25 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x479</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>0x479</t>
+          <t>515</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>515</t>
+          <t>170.04099999999943</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>170.04099999999943</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H76" s="2" t="inlineStr">
         <is>
           <t>sha256:89e1fdf6f94b3a3a9f3488943c2f691ede0159f2325957178723a3ae2807e183:line:550</t>
         </is>
@@ -4236,30 +3854,25 @@
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x489</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>0x489</t>
+          <t>97</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>97</t>
+          <t>900.1354999999976</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>900.1354999999976</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="H77" s="2" t="inlineStr">
         <is>
           <t>sha256:89e1fdf6f94b3a3a9f3488943c2f691ede0159f2325957178723a3ae2807e183:line:1749</t>
         </is>
@@ -4278,30 +3891,25 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x493</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>0x493</t>
+          <t>876</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>876</t>
+          <t>99.75000000000023</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>99.75000000000023</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H78" s="2" t="inlineStr">
         <is>
           <t>sha256:89e1fdf6f94b3a3a9f3488943c2f691ede0159f2325957178723a3ae2807e183:line:313</t>
         </is>
@@ -4320,30 +3928,25 @@
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x494</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>0x494</t>
+          <t>876</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>876</t>
+          <t>99.82800000000225</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>99.82800000000225</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H79" s="2" t="inlineStr">
         <is>
           <t>sha256:89e1fdf6f94b3a3a9f3488943c2f691ede0159f2325957178723a3ae2807e183:line:314</t>
         </is>
@@ -4362,30 +3965,25 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
+          <t>0x499</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>88</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>1000.0679999999988</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="D80" s="2" t="inlineStr">
-        <is>
-          <t>0x499</t>
-        </is>
-      </c>
-      <c r="E80" s="2" t="inlineStr">
-        <is>
-          <t>88</t>
-        </is>
-      </c>
-      <c r="F80" s="2" t="inlineStr">
-        <is>
-          <t>1000.0679999999988</t>
-        </is>
-      </c>
       <c r="G80" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="H80" s="2" t="inlineStr">
         <is>
           <t>sha256:89e1fdf6f94b3a3a9f3488943c2f691ede0159f2325957178723a3ae2807e183:line:2134</t>
         </is>
@@ -4404,30 +4002,25 @@
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x49C</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>0x49C</t>
+          <t>88</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>1000.0639999999947</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>1000.0639999999947</t>
+          <t>13</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="H81" s="2" t="inlineStr">
         <is>
           <t>sha256:89e1fdf6f94b3a3a9f3488943c2f691ede0159f2325957178723a3ae2807e183:line:2135</t>
         </is>
@@ -4446,30 +4039,25 @@
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x4C</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>0x4C</t>
+          <t>2693</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>2693</t>
+          <t>10.007000000001653</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>10.007000000001653</t>
+          <t>15</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="H82" s="2" t="inlineStr">
         <is>
           <t>sha256:cc21dd0ef4b9991918fb1b596346274eebf8c6b5feac7bf9b40f0f8312644626:line:28</t>
         </is>
@@ -4488,30 +4076,25 @@
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x60</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>0x60</t>
+          <t>1347</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>1347</t>
+          <t>19.99400000000051</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>19.99400000000051</t>
+          <t>13</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="H83" s="2" t="inlineStr">
         <is>
           <t>sha256:cc21dd0ef4b9991918fb1b596346274eebf8c6b5feac7bf9b40f0f8312644626:line:29</t>
         </is>
@@ -4530,30 +4113,25 @@
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x63</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>0x63</t>
+          <t>1347</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>1347</t>
+          <t>19.992999999999483</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>19.992999999999483</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H84" s="2" t="inlineStr">
         <is>
           <t>sha256:cc21dd0ef4b9991918fb1b596346274eebf8c6b5feac7bf9b40f0f8312644626:line:30</t>
         </is>
@@ -4572,30 +4150,25 @@
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x110</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>0x110</t>
+          <t>1347</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>1347</t>
+          <t>19.992999999999483</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>19.992999999999483</t>
+          <t>15</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="H85" s="2" t="inlineStr">
         <is>
           <t>sha256:cc21dd0ef4b9991918fb1b596346274eebf8c6b5feac7bf9b40f0f8312644626:line:31</t>
         </is>
@@ -4614,30 +4187,25 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x122</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>0x122</t>
+          <t>586</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>586</t>
+          <t>19.986000000002946</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>19.986000000002946</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H86" s="2" t="inlineStr">
         <is>
           <t>sha256:cc21dd0ef4b9991918fb1b596346274eebf8c6b5feac7bf9b40f0f8312644626:line:42033</t>
         </is>
@@ -4656,30 +4224,25 @@
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x123</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>0x123</t>
+          <t>1347</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>1347</t>
+          <t>19.97599999999977</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>19.97599999999977</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H87" s="2" t="inlineStr">
         <is>
           <t>sha256:cc21dd0ef4b9991918fb1b596346274eebf8c6b5feac7bf9b40f0f8312644626:line:32</t>
         </is>
@@ -4698,30 +4261,25 @@
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x189</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>0x189</t>
+          <t>673</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>673</t>
+          <t>40.00950000000003</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>40.00950000000003</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="H88" s="2" t="inlineStr">
         <is>
           <t>sha256:cc21dd0ef4b9991918fb1b596346274eebf8c6b5feac7bf9b40f0f8312644626:line:92</t>
         </is>
@@ -4740,30 +4298,25 @@
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x1A0</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>0x1A0</t>
+          <t>269</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>269</t>
+          <t>99.94650000000149</t>
         </is>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>99.94650000000149</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H89" s="2" t="inlineStr">
         <is>
           <t>sha256:cc21dd0ef4b9991918fb1b596346274eebf8c6b5feac7bf9b40f0f8312644626:line:192</t>
         </is>
@@ -4782,30 +4335,25 @@
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x220</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>0x220</t>
+          <t>336</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>336</t>
+          <t>80.093999999999</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>80.093999999999</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H90" s="2" t="inlineStr">
         <is>
           <t>sha256:cc21dd0ef4b9991918fb1b596346274eebf8c6b5feac7bf9b40f0f8312644626:line:210</t>
         </is>
@@ -4824,30 +4372,25 @@
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
+          <t>0x265</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>147</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>80.20849999999946</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="D91" s="2" t="inlineStr">
-        <is>
-          <t>0x265</t>
-        </is>
-      </c>
-      <c r="E91" s="2" t="inlineStr">
-        <is>
-          <t>147</t>
-        </is>
-      </c>
-      <c r="F91" s="2" t="inlineStr">
-        <is>
-          <t>80.20849999999946</t>
-        </is>
-      </c>
       <c r="G91" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="H91" s="2" t="inlineStr">
         <is>
           <t>sha256:cc21dd0ef4b9991918fb1b596346274eebf8c6b5feac7bf9b40f0f8312644626:line:42044</t>
         </is>
@@ -4866,30 +4409,25 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x272</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>0x272</t>
+          <t>269</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>269</t>
+          <t>100.11750000000052</t>
         </is>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>100.11750000000052</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H92" s="2" t="inlineStr">
         <is>
           <t>sha256:cc21dd0ef4b9991918fb1b596346274eebf8c6b5feac7bf9b40f0f8312644626:line:211</t>
         </is>
@@ -4908,30 +4446,25 @@
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x283</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>0x283</t>
+          <t>180</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>145.65799999999916</t>
         </is>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>145.65799999999916</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H93" s="2" t="inlineStr">
         <is>
           <t>sha256:cc21dd0ef4b9991918fb1b596346274eebf8c6b5feac7bf9b40f0f8312644626:line:213</t>
         </is>
@@ -4950,30 +4483,25 @@
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x305</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>0x305</t>
+          <t>45</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>600.0260000000006</t>
         </is>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>600.0260000000006</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H94" s="2" t="inlineStr">
         <is>
           <t>sha256:cc21dd0ef4b9991918fb1b596346274eebf8c6b5feac7bf9b40f0f8312644626:line:1041</t>
         </is>
@@ -4992,30 +4520,25 @@
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x457</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>0x457</t>
+          <t>34</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>800.1080000000015</t>
         </is>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>800.1080000000015</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H95" s="2" t="inlineStr">
         <is>
           <t>sha256:cc21dd0ef4b9991918fb1b596346274eebf8c6b5feac7bf9b40f0f8312644626:line:424</t>
         </is>
@@ -5034,30 +4557,25 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x465</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>0x465</t>
+          <t>34</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>800.107999999998</t>
         </is>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>800.107999999998</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H96" s="2" t="inlineStr">
         <is>
           <t>sha256:cc21dd0ef4b9991918fb1b596346274eebf8c6b5feac7bf9b40f0f8312644626:line:425</t>
         </is>
@@ -5076,30 +4594,25 @@
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0x466</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>0x466</t>
+          <t>34</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>800.107999999998</t>
         </is>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>800.107999999998</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H97" s="2" t="inlineStr">
         <is>
           <t>sha256:cc21dd0ef4b9991918fb1b596346274eebf8c6b5feac7bf9b40f0f8312644626:line:426</t>
         </is>
@@ -5118,30 +4631,25 @@
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
+          <t>0x94</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>601</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr">
+        <is>
+          <t>20.001999999999853</t>
+        </is>
+      </c>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D98" s="2" t="inlineStr">
-        <is>
-          <t>0x94</t>
-        </is>
-      </c>
-      <c r="E98" s="2" t="inlineStr">
-        <is>
-          <t>601</t>
-        </is>
-      </c>
-      <c r="F98" s="2" t="inlineStr">
-        <is>
-          <t>20.001999999999853</t>
-        </is>
-      </c>
       <c r="G98" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H98" s="2" t="inlineStr">
         <is>
           <t>sha256:3fbf4569e2b8e97e0b7203996156f63b74a4b817e240498cf11648a812267db3:line:16</t>
         </is>
@@ -5160,30 +4668,25 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0x95</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>0x95</t>
+          <t>1201</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>1201</t>
+          <t>9.998999999999647</t>
         </is>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>9.998999999999647</t>
+          <t>15</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="H99" s="2" t="inlineStr">
         <is>
           <t>sha256:3fbf4569e2b8e97e0b7203996156f63b74a4b817e240498cf11648a812267db3:line:14</t>
         </is>
@@ -5202,30 +4705,25 @@
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
+          <t>0x12B</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>601</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="inlineStr">
+        <is>
+          <t>20.001999999999853</t>
+        </is>
+      </c>
+      <c r="F100" s="2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D100" s="2" t="inlineStr">
-        <is>
-          <t>0x12B</t>
-        </is>
-      </c>
-      <c r="E100" s="2" t="inlineStr">
-        <is>
-          <t>601</t>
-        </is>
-      </c>
-      <c r="F100" s="2" t="inlineStr">
-        <is>
-          <t>20.001999999999853</t>
-        </is>
-      </c>
       <c r="G100" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H100" s="2" t="inlineStr">
         <is>
           <t>sha256:3fbf4569e2b8e97e0b7203996156f63b74a4b817e240498cf11648a812267db3:line:17</t>
         </is>
@@ -5244,30 +4742,25 @@
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
+          <t>0x13A</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>601</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="inlineStr">
+        <is>
+          <t>20.002999999999105</t>
+        </is>
+      </c>
+      <c r="F101" s="2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D101" s="2" t="inlineStr">
-        <is>
-          <t>0x13A</t>
-        </is>
-      </c>
-      <c r="E101" s="2" t="inlineStr">
-        <is>
-          <t>601</t>
-        </is>
-      </c>
-      <c r="F101" s="2" t="inlineStr">
-        <is>
-          <t>20.002999999999105</t>
-        </is>
-      </c>
       <c r="G101" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H101" s="2" t="inlineStr">
         <is>
           <t>sha256:3fbf4569e2b8e97e0b7203996156f63b74a4b817e240498cf11648a812267db3:line:18</t>
         </is>
@@ -5286,30 +4779,25 @@
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0x156</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>0x156</t>
+          <t>601</t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>601</t>
+          <t>20.002999999999993</t>
         </is>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>20.002999999999993</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="H102" s="2" t="inlineStr">
         <is>
           <t>sha256:3fbf4569e2b8e97e0b7203996156f63b74a4b817e240498cf11648a812267db3:line:19</t>
         </is>
@@ -5328,30 +4816,25 @@
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0x180</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>0x180</t>
+          <t>301</t>
         </is>
       </c>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t>301</t>
+          <t>40.00049999999966</t>
         </is>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>40.00049999999966</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="H103" s="2" t="inlineStr">
         <is>
           <t>sha256:3fbf4569e2b8e97e0b7203996156f63b74a4b817e240498cf11648a812267db3:line:20</t>
         </is>
@@ -5370,30 +4853,25 @@
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
+          <t>0x187</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t>99.99199999999853</t>
+        </is>
+      </c>
+      <c r="F104" s="2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D104" s="2" t="inlineStr">
-        <is>
-          <t>0x187</t>
-        </is>
-      </c>
-      <c r="E104" s="2" t="inlineStr">
-        <is>
-          <t>120</t>
-        </is>
-      </c>
-      <c r="F104" s="2" t="inlineStr">
-        <is>
-          <t>99.99199999999853</t>
-        </is>
-      </c>
       <c r="G104" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H104" s="2" t="inlineStr">
         <is>
           <t>sha256:3fbf4569e2b8e97e0b7203996156f63b74a4b817e240498cf11648a812267db3:line:21</t>
         </is>
@@ -5412,30 +4890,25 @@
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
+          <t>0x200</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="E105" s="2" t="inlineStr">
+        <is>
+          <t>79.98599999999989</t>
+        </is>
+      </c>
+      <c r="F105" s="2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D105" s="2" t="inlineStr">
-        <is>
-          <t>0x200</t>
-        </is>
-      </c>
-      <c r="E105" s="2" t="inlineStr">
-        <is>
-          <t>150</t>
-        </is>
-      </c>
-      <c r="F105" s="2" t="inlineStr">
-        <is>
-          <t>79.98599999999989</t>
-        </is>
-      </c>
       <c r="G105" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H105" s="2" t="inlineStr">
         <is>
           <t>sha256:3fbf4569e2b8e97e0b7203996156f63b74a4b817e240498cf11648a812267db3:line:22</t>
         </is>
@@ -5454,30 +4927,25 @@
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
+          <t>0x226</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="E106" s="2" t="inlineStr">
+        <is>
+          <t>79.98600000000033</t>
+        </is>
+      </c>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D106" s="2" t="inlineStr">
-        <is>
-          <t>0x226</t>
-        </is>
-      </c>
-      <c r="E106" s="2" t="inlineStr">
-        <is>
-          <t>150</t>
-        </is>
-      </c>
-      <c r="F106" s="2" t="inlineStr">
-        <is>
-          <t>79.98600000000033</t>
-        </is>
-      </c>
       <c r="G106" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H106" s="2" t="inlineStr">
         <is>
           <t>sha256:3fbf4569e2b8e97e0b7203996156f63b74a4b817e240498cf11648a812267db3:line:150</t>
         </is>
@@ -5496,30 +4964,25 @@
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
+          <t>0x273</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="E107" s="2" t="inlineStr">
+        <is>
+          <t>99.75700000000032</t>
+        </is>
+      </c>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D107" s="2" t="inlineStr">
-        <is>
-          <t>0x273</t>
-        </is>
-      </c>
-      <c r="E107" s="2" t="inlineStr">
-        <is>
-          <t>120</t>
-        </is>
-      </c>
-      <c r="F107" s="2" t="inlineStr">
-        <is>
-          <t>99.75700000000032</t>
-        </is>
-      </c>
       <c r="G107" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H107" s="2" t="inlineStr">
         <is>
           <t>sha256:3fbf4569e2b8e97e0b7203996156f63b74a4b817e240498cf11648a812267db3:line:24</t>
         </is>
@@ -5538,30 +5001,25 @@
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
+          <t>0x275</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>75</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="inlineStr">
+        <is>
+          <t>160.0215000000009</t>
+        </is>
+      </c>
+      <c r="F108" s="2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D108" s="2" t="inlineStr">
-        <is>
-          <t>0x275</t>
-        </is>
-      </c>
-      <c r="E108" s="2" t="inlineStr">
-        <is>
-          <t>75</t>
-        </is>
-      </c>
-      <c r="F108" s="2" t="inlineStr">
-        <is>
-          <t>160.0215000000009</t>
-        </is>
-      </c>
       <c r="G108" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H108" s="2" t="inlineStr">
         <is>
           <t>sha256:3fbf4569e2b8e97e0b7203996156f63b74a4b817e240498cf11648a812267db3:line:286</t>
         </is>
@@ -5580,30 +5038,25 @@
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
+          <t>0x280</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="E109" s="2" t="inlineStr">
+        <is>
+          <t>120.01099999999987</t>
+        </is>
+      </c>
+      <c r="F109" s="2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D109" s="2" t="inlineStr">
-        <is>
-          <t>0x280</t>
-        </is>
-      </c>
-      <c r="E109" s="2" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="F109" s="2" t="inlineStr">
-        <is>
-          <t>120.01099999999987</t>
-        </is>
-      </c>
       <c r="G109" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H109" s="2" t="inlineStr">
         <is>
           <t>sha256:3fbf4569e2b8e97e0b7203996156f63b74a4b817e240498cf11648a812267db3:line:28</t>
         </is>
@@ -5622,30 +5075,25 @@
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
+          <t>0x49A</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="inlineStr">
+        <is>
+          <t>799.8259999999999</t>
+        </is>
+      </c>
+      <c r="F110" s="2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D110" s="2" t="inlineStr">
-        <is>
-          <t>0x49A</t>
-        </is>
-      </c>
-      <c r="E110" s="2" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="F110" s="2" t="inlineStr">
-        <is>
-          <t>799.8259999999999</t>
-        </is>
-      </c>
       <c r="G110" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H110" s="2" t="inlineStr">
         <is>
           <t>sha256:3fbf4569e2b8e97e0b7203996156f63b74a4b817e240498cf11648a812267db3:line:699</t>
         </is>
@@ -5664,30 +5112,25 @@
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
+          <t>0x49B</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E111" s="2" t="inlineStr">
+        <is>
+          <t>800.0779999999996</t>
+        </is>
+      </c>
+      <c r="F111" s="2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D111" s="2" t="inlineStr">
-        <is>
-          <t>0x49B</t>
-        </is>
-      </c>
-      <c r="E111" s="2" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="F111" s="2" t="inlineStr">
-        <is>
-          <t>800.0779999999996</t>
-        </is>
-      </c>
       <c r="G111" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H111" s="2" t="inlineStr">
         <is>
           <t>sha256:3fbf4569e2b8e97e0b7203996156f63b74a4b817e240498cf11648a812267db3:line:710</t>
         </is>

</xml_diff>

<commit_message>
Publish full raw-trace findings and corrected torque/current candidates
</commit_message>
<xml_diff>
--- a/reports/Zeekr_X_CAN_Matrix_EN.xlsx
+++ b/reports/Zeekr_X_CAN_Matrix_EN.xlsx
@@ -17,8 +17,9 @@
     <sheet name="BECM" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="DC-DC" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Stalk switch" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Bridge evidence" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Legend" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Drive role hypotheses" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Bridge evidence" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Legend" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -211,7 +212,22 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="T11" displayName="T11" ref="A1:G111" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="T11" displayName="T11" ref="A1:F19" headerRowCount="1">
+  <autoFilter ref="A1:F19"/>
+  <tableColumns count="6">
+    <tableColumn id="1" name="Axle"/>
+    <tableColumn id="2" name="Role"/>
+    <tableColumn id="3" name="Field"/>
+    <tableColumn id="4" name="Status"/>
+    <tableColumn id="5" name="Physical_Nm_Confirmed"/>
+    <tableColumn id="6" name="Evidence"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="T12" displayName="T12" ref="A1:G111" headerRowCount="1">
   <autoFilter ref="A1:G111"/>
   <tableColumns count="7">
     <tableColumn id="1" name="Experiment"/>
@@ -226,8 +242,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="T12" displayName="T12" ref="A1:B6" headerRowCount="1">
+<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="T13" displayName="T13" ref="A1:B6" headerRowCount="1">
   <autoFilter ref="A1:B6"/>
   <tableColumns count="2">
     <tableColumn id="1" name="Status"/>
@@ -269,8 +285,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="T4" displayName="T4" ref="A1:U36" headerRowCount="1">
-  <autoFilter ref="A1:U36"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="T4" displayName="T4" ref="A1:U42" headerRowCount="1">
+  <autoFilter ref="A1:U42"/>
   <tableColumns count="21">
     <tableColumn id="1" name="Bus"/>
     <tableColumn id="2" name="CAN_ID"/>
@@ -761,12 +777,12 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>41</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>4 confirmed VIN layout fields, 29 candidates, 2 unknown fields.</t>
+          <t>4 confirmed VIN layout fields, 35 candidates, 2 unknown fields. No new physical torque calibration.</t>
         </is>
       </c>
     </row>
@@ -1017,6 +1033,639 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="63" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="37" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Axle</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Physical_Nm_Confirmed</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="45" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>RearDrive</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>request</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>VCU 0x04B MSB0 12/16; 0.25*raw-8190</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>CANDIDATE</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>reports/full_raw_review_20261017.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="45" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>RearDrive</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>current_or_actual</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>0x04C MSB0 8/14; raw-8188</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>CANDIDATE</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>reports/full_raw_review_20261017.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="45" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>RearDrive</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>positive_limit</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>0x04C MSB0 40/12; 4*(raw-2047)</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>CANDIDATE</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>reports/full_raw_review_20261017.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="45" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>RearDrive</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>negative_limit</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>0x04C MSB0 52/12; complementary to positive field</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>CANDIDATE</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>reports/full_raw_review_20261017.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="45" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>RearDrive</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>mode</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>reports/full_raw_review_20261017.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="45" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>RearDrive</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>enable</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>reports/full_raw_review_20261017.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="45" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>RearDrive</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>speed</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>reports/full_raw_review_20261017.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="45" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>RearDrive</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>DC_current</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>0x063 MSB0 2/14; 0.1*raw-818.8 candidate</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>CANDIDATE</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>reports/full_raw_review_20261017.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="45" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>RearDrive</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>fault</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>reports/full_raw_review_20261017.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="45" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>FrontDrive</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>request</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>VCU 0x050 MSB0 2/14; raw-8188</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>CANDIDATE</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>reports/full_raw_review_20261017.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="45" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>FrontDrive</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>current_or_actual</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>0x095 MSB0 18/14; raw-8188</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>CANDIDATE</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>reports/full_raw_review_20261017.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="45" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>FrontDrive</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>positive_limit</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>0x13A MSB0 0/14; raw-8188</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>CANDIDATE</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>reports/full_raw_review_20261017.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="45" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>FrontDrive</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>negative_limit</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>0x13A MSB0 16/14; complementary to positive field</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>CANDIDATE</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>reports/full_raw_review_20261017.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="45" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>FrontDrive</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>mode</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>reports/full_raw_review_20261017.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="45" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>FrontDrive</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>enable</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>reports/full_raw_review_20261017.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="45" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>FrontDrive</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>speed</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>0x180 MSB0 16/16; raw*0.5, physical rotation units unverified</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>CANDIDATE</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>reports/full_raw_review_20261017.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="45" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>FrontDrive</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>DC_current</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>0x13A MSB0 50/14; 0.1*raw-818.8 candidate</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>CANDIDATE</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>reports/full_raw_review_20261017.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="45" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>FrontDrive</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>fault</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>reports/full_raw_review_20261017.md</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -5144,7 +5793,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5893,9 +6542,9 @@
           <t>0x4B</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>CANDIDATE</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -5940,9 +6589,9 @@
           <t>0x4C</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>CANDIDATE</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -6175,9 +6824,9 @@
           <t>0x63</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>CANDIDATE</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -12048,7 +12697,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U36"/>
+  <dimension ref="A1:U42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -12890,7 +13539,7 @@
       </c>
       <c r="U8" s="2" t="inlineStr">
         <is>
-          <t>Historical diagnostic labels do not establish axle identity. Candidate formulas require independent validation.</t>
+          <t>Rejected as a universal high-load decoder: signed12 wraps in dynamic traces; retained as a historical low-current candidate. See reports/full_raw_review_20261017.md.</t>
         </is>
       </c>
     </row>
@@ -13372,7 +14021,7 @@
       </c>
       <c r="U14" s="2" t="inlineStr">
         <is>
-          <t>Historical diagnostic labels do not establish axle identity. Candidate formulas require independent validation.</t>
+          <t>Complementary amplitude candidate, not an independently verified positive torque limit. Six pair-sum exceptions.</t>
         </is>
       </c>
     </row>
@@ -13463,7 +14112,7 @@
       </c>
       <c r="U15" s="2" t="inlineStr">
         <is>
-          <t>Historical diagnostic labels do not establish axle identity. Candidate formulas require independent validation.</t>
+          <t>Complementary to A except six frames; not an independently verified regeneration limit.</t>
         </is>
       </c>
     </row>
@@ -14544,7 +15193,7 @@
       </c>
       <c r="U26" s="2" t="inlineStr">
         <is>
-          <t>Historical diagnostic labels do not establish axle identity. Candidate formulas require independent validation.</t>
+          <t>Dynamic interpretation unsupported: 135 comparisons showed constant realtime field while diagnostic voltage varied.</t>
         </is>
       </c>
     </row>
@@ -15479,6 +16128,528 @@
       <c r="U36" s="2" t="inlineStr">
         <is>
           <t>VIN layout verified against owner-provided identifier; identifier and payload omitted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="45" customHeight="1">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Propulsion_CAN</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>0x4B</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>RearTorqueRequest_raw_candidate</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>big</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>-8190</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr"/>
+      <c r="K37" s="5" t="inlineStr">
+        <is>
+          <t>CANDIDATE</t>
+        </is>
+      </c>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>MSB0_LINEAR</t>
+        </is>
+      </c>
+      <c r="M37" s="2" t="inlineStr"/>
+      <c r="N37" s="2" t="inlineStr"/>
+      <c r="O37" s="2" t="inlineStr">
+        <is>
+          <t>VCU</t>
+        </is>
+      </c>
+      <c r="P37" s="2" t="inlineStr"/>
+      <c r="Q37" s="2" t="inlineStr"/>
+      <c r="R37" s="2" t="inlineStr">
+        <is>
+          <t>sha256:152e54ebf741020ff09d6b29235c52113c7dbaa01c2247931b42795b9a2adf68:line:11;sha256:2a800f01f942668fe425dde9cc08555a5d2a37323aacb9f994eb21455318b2ea:line:5;sha256:53dfbbc0c579fb710a53ab23f9539640d4494b6b14802cf6aa13afd7f660af08:line:23</t>
+        </is>
+      </c>
+      <c r="S37" s="2" t="inlineStr">
+        <is>
+          <t>SOURCE_AWARE_RAW_REVIEW_FROZEN_FIELD_AND_COMPETING_MODEL_TEST</t>
+        </is>
+      </c>
+      <c r="T37" s="2" t="inlineStr">
+        <is>
+          <t>Source recordings retained by maintainer; not included in public snapshot</t>
+        </is>
+      </c>
+      <c r="U37" s="2" t="inlineStr">
+        <is>
+          <t>Training: calm acceleration structural window; lower-bit and physical scale boundaries remain uncertain. Display units are provisional; unit deliberately blank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="45" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Propulsion_CAN</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>0x4C</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>RearTorqueFeedback_raw_candidate</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>big</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>-8188</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr"/>
+      <c r="K38" s="5" t="inlineStr">
+        <is>
+          <t>CANDIDATE</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>MSB0_LINEAR</t>
+        </is>
+      </c>
+      <c r="M38" s="2" t="inlineStr"/>
+      <c r="N38" s="2" t="inlineStr"/>
+      <c r="O38" s="2" t="inlineStr">
+        <is>
+          <t>RearDrive</t>
+        </is>
+      </c>
+      <c r="P38" s="2" t="inlineStr"/>
+      <c r="Q38" s="2" t="inlineStr"/>
+      <c r="R38" s="2" t="inlineStr">
+        <is>
+          <t>sha256:152e54ebf741020ff09d6b29235c52113c7dbaa01c2247931b42795b9a2adf68:line:36;sha256:2a800f01f942668fe425dde9cc08555a5d2a37323aacb9f994eb21455318b2ea:line:42;sha256:53dfbbc0c579fb710a53ab23f9539640d4494b6b14802cf6aa13afd7f660af08:line:18</t>
+        </is>
+      </c>
+      <c r="S38" s="2" t="inlineStr">
+        <is>
+          <t>SOURCE_AWARE_RAW_REVIEW_FROZEN_FIELD_AND_COMPETING_MODEL_TEST</t>
+        </is>
+      </c>
+      <c r="T38" s="2" t="inlineStr">
+        <is>
+          <t>Source recordings retained by maintainer; not included in public snapshot</t>
+        </is>
+      </c>
+      <c r="U38" s="2" t="inlineStr">
+        <is>
+          <t>Tracks request in several regimes; not numerically equal to E304; not confirmed actual shaft torque. Display units are provisional; unit deliberately blank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="45" customHeight="1">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Propulsion_CAN</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>0x4C</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>RearTorqueBoundA_raw_candidate</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>big</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>-8188</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr"/>
+      <c r="K39" s="5" t="inlineStr">
+        <is>
+          <t>CANDIDATE</t>
+        </is>
+      </c>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>MSB0_LINEAR</t>
+        </is>
+      </c>
+      <c r="M39" s="2" t="inlineStr"/>
+      <c r="N39" s="2" t="inlineStr"/>
+      <c r="O39" s="2" t="inlineStr">
+        <is>
+          <t>RearDrive</t>
+        </is>
+      </c>
+      <c r="P39" s="2" t="inlineStr"/>
+      <c r="Q39" s="2" t="inlineStr"/>
+      <c r="R39" s="2" t="inlineStr">
+        <is>
+          <t>sha256:152e54ebf741020ff09d6b29235c52113c7dbaa01c2247931b42795b9a2adf68:line:36;sha256:2a800f01f942668fe425dde9cc08555a5d2a37323aacb9f994eb21455318b2ea:line:42;sha256:53dfbbc0c579fb710a53ab23f9539640d4494b6b14802cf6aa13afd7f660af08:line:18</t>
+        </is>
+      </c>
+      <c r="S39" s="2" t="inlineStr">
+        <is>
+          <t>SOURCE_AWARE_RAW_REVIEW_FROZEN_FIELD_AND_COMPETING_MODEL_TEST</t>
+        </is>
+      </c>
+      <c r="T39" s="2" t="inlineStr">
+        <is>
+          <t>Source recordings retained by maintainer; not included in public snapshot</t>
+        </is>
+      </c>
+      <c r="U39" s="2" t="inlineStr">
+        <is>
+          <t>Complementary pair; scale factor 4 is exploratory comparison to request, not Nm. Display units are provisional; unit deliberately blank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="45" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Propulsion_CAN</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>0x4C</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>RearTorqueBoundB_raw_candidate</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>big</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>-8188</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr"/>
+      <c r="K40" s="5" t="inlineStr">
+        <is>
+          <t>CANDIDATE</t>
+        </is>
+      </c>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>MSB0_LINEAR</t>
+        </is>
+      </c>
+      <c r="M40" s="2" t="inlineStr"/>
+      <c r="N40" s="2" t="inlineStr"/>
+      <c r="O40" s="2" t="inlineStr">
+        <is>
+          <t>RearDrive</t>
+        </is>
+      </c>
+      <c r="P40" s="2" t="inlineStr"/>
+      <c r="Q40" s="2" t="inlineStr"/>
+      <c r="R40" s="2" t="inlineStr">
+        <is>
+          <t>sha256:152e54ebf741020ff09d6b29235c52113c7dbaa01c2247931b42795b9a2adf68:line:36;sha256:2a800f01f942668fe425dde9cc08555a5d2a37323aacb9f994eb21455318b2ea:line:42;sha256:53dfbbc0c579fb710a53ab23f9539640d4494b6b14802cf6aa13afd7f660af08:line:18</t>
+        </is>
+      </c>
+      <c r="S40" s="2" t="inlineStr">
+        <is>
+          <t>SOURCE_AWARE_RAW_REVIEW_FROZEN_FIELD_AND_COMPETING_MODEL_TEST</t>
+        </is>
+      </c>
+      <c r="T40" s="2" t="inlineStr">
+        <is>
+          <t>Source recordings retained by maintainer; not included in public snapshot</t>
+        </is>
+      </c>
+      <c r="U40" s="2" t="inlineStr">
+        <is>
+          <t>Not an independent negative limit: complementary to A in all but five observed frames. Display units are provisional; unit deliberately blank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="45" customHeight="1">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Propulsion_CAN</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>0x63</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>RearDCCurrent_raw_candidate</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>big</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>0.1</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>-818.8</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr"/>
+      <c r="K41" s="5" t="inlineStr">
+        <is>
+          <t>CANDIDATE</t>
+        </is>
+      </c>
+      <c r="L41" s="2" t="inlineStr">
+        <is>
+          <t>MSB0_LINEAR</t>
+        </is>
+      </c>
+      <c r="M41" s="2" t="inlineStr"/>
+      <c r="N41" s="2" t="inlineStr"/>
+      <c r="O41" s="2" t="inlineStr">
+        <is>
+          <t>RearDrive</t>
+        </is>
+      </c>
+      <c r="P41" s="2" t="inlineStr"/>
+      <c r="Q41" s="2" t="inlineStr"/>
+      <c r="R41" s="2" t="inlineStr">
+        <is>
+          <t>sha256:152e54ebf741020ff09d6b29235c52113c7dbaa01c2247931b42795b9a2adf68:line:65;sha256:2a800f01f942668fe425dde9cc08555a5d2a37323aacb9f994eb21455318b2ea:line:6;sha256:53dfbbc0c579fb710a53ab23f9539640d4494b6b14802cf6aa13afd7f660af08:line:46</t>
+        </is>
+      </c>
+      <c r="S41" s="2" t="inlineStr">
+        <is>
+          <t>SOURCE_AWARE_RAW_REVIEW_FROZEN_FIELD_AND_COMPETING_MODEL_TEST</t>
+        </is>
+      </c>
+      <c r="T41" s="2" t="inlineStr">
+        <is>
+          <t>Source recordings retained by maintainer; not included in public snapshot</t>
+        </is>
+      </c>
+      <c r="U41" s="2" t="inlineStr">
+        <is>
+          <t>Electrical-flow hypothesis; rear+front relation depends on unresolved BECM decoding. A not physically confirmed. Display units are provisional; unit deliberately blank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="45" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Propulsion_CAN</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>0x143</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>BatteryCurrent_Word16_alternative</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>big</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>0.1</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>-4914.8</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr"/>
+      <c r="K42" s="5" t="inlineStr">
+        <is>
+          <t>CANDIDATE</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>MSB0_LINEAR</t>
+        </is>
+      </c>
+      <c r="M42" s="2" t="inlineStr"/>
+      <c r="N42" s="2" t="inlineStr"/>
+      <c r="O42" s="2" t="inlineStr">
+        <is>
+          <t>BECM</t>
+        </is>
+      </c>
+      <c r="P42" s="2" t="inlineStr"/>
+      <c r="Q42" s="2" t="inlineStr"/>
+      <c r="R42" s="2" t="inlineStr">
+        <is>
+          <t>sha256:152e54ebf741020ff09d6b29235c52113c7dbaa01c2247931b42795b9a2adf68:line:18;sha256:2a800f01f942668fe425dde9cc08555a5d2a37323aacb9f994eb21455318b2ea:line:31;sha256:53dfbbc0c579fb710a53ab23f9539640d4494b6b14802cf6aa13afd7f660af08:line:65</t>
+        </is>
+      </c>
+      <c r="S42" s="2" t="inlineStr">
+        <is>
+          <t>SOURCE_AWARE_RAW_REVIEW_FROZEN_FIELD_AND_COMPETING_MODEL_TEST</t>
+        </is>
+      </c>
+      <c r="T42" s="2" t="inlineStr">
+        <is>
+          <t>Source recordings retained by maintainer; not included in public snapshot</t>
+        </is>
+      </c>
+      <c r="U42" s="2" t="inlineStr">
+        <is>
+          <t>Exploratory full-word alternative to signed12. High-load physical calibration and bit boundaries are unresolved.</t>
         </is>
       </c>
     </row>
@@ -15568,9 +16739,9 @@
           <t>0x4C</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>CANDIDATE</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -15662,9 +16833,9 @@
           <t>0x63</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>CANDIDATE</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -17363,9 +18534,9 @@
           <t>0x4B</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>CANDIDATE</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">

</xml_diff>